<commit_message>
Daily slate 2026-06-02 [auto]
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-05-31.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-05-31.xlsx
@@ -471,16 +471,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="E2" t="n">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="F2" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="G2" t="n">
-        <v>52.2</v>
+        <v>53.3</v>
       </c>
     </row>
     <row r="3">
@@ -529,16 +529,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="E4" t="n">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="F4" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G4" t="n">
-        <v>49.3</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5">
@@ -558,16 +558,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="E5" t="n">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="F5" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="G5" t="n">
-        <v>48.1</v>
+        <v>49.3</v>
       </c>
     </row>
     <row r="6">
@@ -616,16 +616,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="E7" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G7" t="n">
-        <v>57.9</v>
+        <v>59.1</v>
       </c>
     </row>
     <row r="8">
@@ -732,16 +732,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>996</v>
+        <v>1046</v>
       </c>
       <c r="E11" t="n">
-        <v>623</v>
+        <v>652</v>
       </c>
       <c r="F11" t="n">
-        <v>373</v>
+        <v>394</v>
       </c>
       <c r="G11" t="n">
-        <v>62.6</v>
+        <v>62.3</v>
       </c>
     </row>
     <row r="12">
@@ -761,16 +761,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="E12" t="n">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="F12" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G12" t="n">
-        <v>72</v>
+        <v>72.2</v>
       </c>
     </row>
     <row r="13">
@@ -819,16 +819,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>362</v>
+        <v>386</v>
       </c>
       <c r="E14" t="n">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="F14" t="n">
-        <v>265</v>
+        <v>285</v>
       </c>
       <c r="G14" t="n">
-        <v>26.8</v>
+        <v>26.2</v>
       </c>
     </row>
     <row r="15">
@@ -848,16 +848,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>437</v>
+        <v>453</v>
       </c>
       <c r="E15" t="n">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="F15" t="n">
-        <v>347</v>
+        <v>360</v>
       </c>
       <c r="G15" t="n">
-        <v>20.6</v>
+        <v>20.5</v>
       </c>
     </row>
     <row r="16">
@@ -906,16 +906,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>4233</v>
+        <v>4439</v>
       </c>
       <c r="E17" t="n">
-        <v>943</v>
+        <v>994</v>
       </c>
       <c r="F17" t="n">
-        <v>3290</v>
+        <v>3445</v>
       </c>
       <c r="G17" t="n">
-        <v>22.3</v>
+        <v>22.4</v>
       </c>
     </row>
   </sheetData>
@@ -1474,16 +1474,16 @@
         <v>96</v>
       </c>
       <c r="D7" t="n">
-        <v>62.6</v>
+        <v>62.3</v>
       </c>
       <c r="E7" t="n">
-        <v>996</v>
+        <v>1046</v>
       </c>
       <c r="F7" t="n">
-        <v>72</v>
+        <v>72.2</v>
       </c>
       <c r="G7" t="n">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="H7" t="n">
         <v>42.2</v>
@@ -1492,16 +1492,16 @@
         <v>102</v>
       </c>
       <c r="J7" t="n">
-        <v>26.8</v>
+        <v>26.2</v>
       </c>
       <c r="K7" t="n">
-        <v>362</v>
+        <v>386</v>
       </c>
       <c r="L7" t="n">
-        <v>20.6</v>
+        <v>20.5</v>
       </c>
       <c r="M7" t="n">
-        <v>437</v>
+        <v>453</v>
       </c>
       <c r="N7" t="n">
         <v>26.3</v>
@@ -1510,22 +1510,22 @@
         <v>114</v>
       </c>
       <c r="P7" t="n">
-        <v>22.3</v>
+        <v>22.4</v>
       </c>
       <c r="Q7" t="n">
-        <v>4233</v>
+        <v>4439</v>
       </c>
       <c r="R7" t="n">
-        <v>52.2</v>
+        <v>53.3</v>
       </c>
       <c r="S7" t="n">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="T7" t="n">
-        <v>49.3</v>
+        <v>50</v>
       </c>
       <c r="U7" t="n">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="V7" t="n">
         <v>63.1</v>
@@ -1546,16 +1546,16 @@
         <v>119</v>
       </c>
       <c r="AB7" t="n">
-        <v>48.1</v>
+        <v>49.3</v>
       </c>
       <c r="AC7" t="n">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="AD7" t="n">
-        <v>57.9</v>
+        <v>59.1</v>
       </c>
       <c r="AE7" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="AF7" t="n">
         <v>0</v>

</xml_diff>